<commit_message>
addional coverage to negative cases
</commit_message>
<xml_diff>
--- a/dummyData.xlsx
+++ b/dummyData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://endava-my.sharepoint.com/personal/dumitru_plamadeala_endava_com/Documents/Desktop/NSG-MRE-SCRIPT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:1_{7A7F1FDD-8B04-4441-BDD8-5B14B5359350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73F57A76-7A39-40D0-A210-DA14EF88F087}"/>
+  <xr:revisionPtr revIDLastSave="89" documentId="13_ncr:1_{7A7F1FDD-8B04-4441-BDD8-5B14B5359350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24F5BD89-0ACB-412F-BD2E-C2AC7F3A5FE9}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{66E66D74-05FB-4940-AC6B-6DDB17CE64BE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="96">
   <si>
     <t>Action</t>
   </si>
@@ -105,9 +105,6 @@
     <t>10.28.32.14</t>
   </si>
   <si>
-    <t>10.28.32.15</t>
-  </si>
-  <si>
     <t>10.10.10.10</t>
   </si>
   <si>
@@ -319,15 +316,6 @@
   </si>
   <si>
     <t>440-445;</t>
-  </si>
-  <si>
-    <t>10.28.32.16; 10.28.32.16;</t>
-  </si>
-  <si>
-    <t>SAP_GW_501</t>
-  </si>
-  <si>
-    <t>10.28.32.14;</t>
   </si>
   <si>
     <t>SAP-NEW_1</t>
@@ -779,7 +767,7 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>1</v>
@@ -806,7 +794,7 @@
         <v>9</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>11</v>
@@ -820,37 +808,37 @@
         <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H2" s="2">
         <v>100</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -858,37 +846,37 @@
         <v>13</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H3" s="2">
         <v>101</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -896,37 +884,37 @@
         <v>13</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="H4" s="2">
         <v>102</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -934,37 +922,37 @@
         <v>13</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="H5" s="2">
         <v>103</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="72" x14ac:dyDescent="0.3">
@@ -972,37 +960,37 @@
         <v>13</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H6" s="2">
         <v>104</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="N6" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="72" x14ac:dyDescent="0.3">
@@ -1010,37 +998,37 @@
         <v>13</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H7" s="2">
         <v>105</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="N7" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="72" x14ac:dyDescent="0.3">
@@ -1048,17 +1036,17 @@
         <v>13</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G8" s="2">
         <v>22</v>
@@ -1067,18 +1055,18 @@
         <v>107</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="N8" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1089,7 +1077,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E6699DB-F1B6-43A3-AC90-D8377FCA7CDF}">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr defaultColWidth="21.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.44140625" bestFit="1" customWidth="1"/>
@@ -1115,7 +1103,7 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>1</v>
@@ -1142,7 +1130,7 @@
         <v>9</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>11</v>
@@ -1162,13 +1150,13 @@
         <v>20</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G2" s="2">
         <v>22</v>
@@ -1177,18 +1165,18 @@
         <v>1000</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1199,36 +1187,36 @@
         <v>15</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H3" s="2">
         <v>1001</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1239,36 +1227,36 @@
         <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H4" s="2">
         <v>1002</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -1282,33 +1270,33 @@
         <v>21</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="H5" s="2">
         <v>1003</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -1316,137 +1304,139 @@
         <v>13</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>96</v>
+        <v>84</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>95</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="H6" s="2">
-        <v>1004</v>
+      <c r="G6" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="H6" s="4">
+        <v>1005</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L6" s="2"/>
-      <c r="M6" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>42</v>
-      </c>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="E7" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G7" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="H7" s="4">
+        <v>1006</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="H7" s="4">
-        <v>1005</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>98</v>
+        <v>18</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="H8" s="4">
-        <v>1006</v>
+        <v>59</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" s="2">
+        <v>2001</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
+        <v>10</v>
+      </c>
+      <c r="L8" s="2">
+        <v>60</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="9" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>27</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H9" s="2">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>35</v>
@@ -1462,49 +1452,7 @@
         <v>47</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H10" s="2">
-        <v>2002</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="L10" s="2">
-        <v>60</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1768,20 +1716,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="28b9e305-6540-4a8f-adff-9abbf67a9457" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="28b9e305-6540-4a8f-adff-9abbf67a9457" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1804,14 +1752,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D9D5B3E-6F96-42BC-A5EA-BACFD70EAC33}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{895FB154-B56A-495E-8783-E6DB4BCA3C3E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -1828,6 +1768,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D9D5B3E-6F96-42BC-A5EA-BACFD70EAC33}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{94d26a2e-8b36-46ca-a6cf-bdb96546be89}" enabled="1" method="Privileged" siteId="{0b3fc178-b730-4e8b-9843-e81259237b77}" contentBits="0" removed="0"/>

</xml_diff>

<commit_message>
improvement on idempotency principle
</commit_message>
<xml_diff>
--- a/dummyData.xlsx
+++ b/dummyData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://endava-my.sharepoint.com/personal/dumitru_plamadeala_endava_com/Documents/Desktop/NSG-MRE-SCRIPT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="89" documentId="13_ncr:1_{7A7F1FDD-8B04-4441-BDD8-5B14B5359350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24F5BD89-0ACB-412F-BD2E-C2AC7F3A5FE9}"/>
+  <xr:revisionPtr revIDLastSave="92" documentId="13_ncr:1_{7A7F1FDD-8B04-4441-BDD8-5B14B5359350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5AF8E83C-945C-43EB-9CEE-8D42CC1C6E23}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{66E66D74-05FB-4940-AC6B-6DDB17CE64BE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{66E66D74-05FB-4940-AC6B-6DDB17CE64BE}"/>
   </bookViews>
   <sheets>
     <sheet name="CoreRules" sheetId="1" r:id="rId1"/>
@@ -48,9 +48,6 @@
     <t>Source Host Name (DNS) FQDN</t>
   </si>
   <si>
-    <t>Destionation IP adress / Subnet / Range IP</t>
-  </si>
-  <si>
     <t>Destination Protocol</t>
   </si>
   <si>
@@ -201,9 +198,6 @@
     <t>CI60</t>
   </si>
   <si>
-    <t>Source IP adress / Subnet / Range IP</t>
-  </si>
-  <si>
     <t>hostname1.porche.com</t>
   </si>
   <si>
@@ -325,6 +319,12 @@
   </si>
   <si>
     <t>10.28.32.112</t>
+  </si>
+  <si>
+    <t>Source IP address / Subnet / Range IP</t>
+  </si>
+  <si>
+    <t>Destination IP address / Subnet / Range IP</t>
   </si>
 </sst>
 </file>
@@ -767,286 +767,286 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>54</v>
+        <v>94</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="3" t="s">
-        <v>9</v>
-      </c>
       <c r="L1" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H2" s="2">
         <v>100</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H3" s="2">
         <v>101</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="N3" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="H4" s="2">
         <v>102</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="H5" s="2">
         <v>103</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H6" s="2">
         <v>104</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="H7" s="2">
         <v>105</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>90</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G8" s="2">
         <v>22</v>
@@ -1055,18 +1055,18 @@
         <v>107</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1103,60 +1103,60 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>54</v>
+        <v>94</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="3" t="s">
-        <v>9</v>
-      </c>
       <c r="L1" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>11</v>
-      </c>
-      <c r="N1" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="C2" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G2" s="2">
         <v>22</v>
@@ -1165,171 +1165,171 @@
         <v>1000</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="61.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H3" s="2">
         <v>1001</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H4" s="2">
         <v>1002</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="H5" s="2">
         <v>1003</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H6" s="4">
         <v>1005</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
@@ -1337,35 +1337,35 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H7" s="4">
         <v>1006</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
@@ -1373,86 +1373,86 @@
     </row>
     <row r="8" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H8" s="2">
         <v>2001</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L8" s="2">
         <v>60</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H9" s="2">
         <v>2002</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J9" s="2"/>
       <c r="K9" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L9" s="2">
         <v>60</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1463,6 +1463,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="28b9e305-6540-4a8f-adff-9abbf67a9457" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010015ACE1AB7268A5458AC0B83055E08635" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e052996763366cd34d38aa15b997ceb6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="ca2eab16-4a02-4618-8f5f-796fd976fad0" xmlns:ns4="28b9e305-6540-4a8f-adff-9abbf67a9457" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9eb40f27300348baafeb0af7684f4cc8" ns3:_="" ns4:_="">
     <xsd:import namespace="ca2eab16-4a02-4618-8f5f-796fd976fad0"/>
@@ -1715,38 +1732,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="28b9e305-6540-4a8f-adff-9abbf67a9457" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C515B5D-F162-4360-8913-11D1CBEB4EBF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D9D5B3E-6F96-42BC-A5EA-BACFD70EAC33}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ca2eab16-4a02-4618-8f5f-796fd976fad0"/>
-    <ds:schemaRef ds:uri="28b9e305-6540-4a8f-adff-9abbf67a9457"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1769,9 +1758,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D9D5B3E-6F96-42BC-A5EA-BACFD70EAC33}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C515B5D-F162-4360-8913-11D1CBEB4EBF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ca2eab16-4a02-4618-8f5f-796fd976fad0"/>
+    <ds:schemaRef ds:uri="28b9e305-6540-4a8f-adff-9abbf67a9457"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>